<commit_message>
Remove bogus 'First Level Magic-User Spells' entry from Illusionist Level 7
That row was a PDF section heading accidentally captured as a spell name.
Illusionist Level 7 now has the correct 5 spells only.

https://claude.ai/code/session_01WowweCqYWM9qAZzzqXzUbu
</commit_message>
<xml_diff>
--- a/AD&D 1e Mage Illusionist Spells.xlsx
+++ b/AD&D 1e Mage Illusionist Spells.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Spell List" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend &amp; Notes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Master Spell List" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Legend &amp; Notes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Master Spell List'!$A$1:$I$261</definedName>
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I261"/>
+  <dimension ref="A1:I260"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -12226,51 +12226,6 @@
       <c r="I260" s="4" t="inlineStr">
         <is>
           <t>Special</t>
-        </is>
-      </c>
-    </row>
-    <row r="261">
-      <c r="A261" s="8" t="inlineStr">
-        <is>
-          <t>Illusionist</t>
-        </is>
-      </c>
-      <c r="B261" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="C261" s="4" t="inlineStr">
-        <is>
-          <t>First Level Magic-User Spells</t>
-        </is>
-      </c>
-      <c r="D261" s="4" t="inlineStr">
-        <is>
-          <t>Various</t>
-        </is>
-      </c>
-      <c r="E261" s="4" t="inlineStr">
-        <is>
-          <t>Gain 4 first-level MU spells at 14th level, +1 per level thereafter. Choose from PHB list.</t>
-        </is>
-      </c>
-      <c r="F261" s="5" t="inlineStr">
-        <is>
-          <t>Special</t>
-        </is>
-      </c>
-      <c r="G261" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H261" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I261" s="4" t="inlineStr">
-        <is>
-          <t>Per spell</t>
         </is>
       </c>
     </row>

</xml_diff>